<commit_message>
BOM Creation / Review
Created Digikey BOM for Transmitter.
Reviewed and fixed mistakes in Receiver BOM
</commit_message>
<xml_diff>
--- a/Hardware-Designing/_Documents/Deliverables-(Receiver)/BOM/Martin_BOM_DigiKey.xlsx
+++ b/Hardware-Designing/_Documents/Deliverables-(Receiver)/BOM/Martin_BOM_DigiKey.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\Martin_Smith\Hardware-Designing\_Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Temporary\MartinS\Martin_Smith\Hardware-Designing\_Documents\Deliverables-(Receiver)\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="255">
   <si>
     <t>S. No.</t>
   </si>
@@ -91,9 +91,6 @@
   </si>
   <si>
     <t>Mouser</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>The only available vibration sensor on digikey</t>
@@ -794,7 +791,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="4">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -1772,6 +1769,7 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="16" fillId="6" borderId="0" xfId="3" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1814,7 +1812,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="6" borderId="0" xfId="3" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Check Cell" xfId="2" builtinId="23"/>
@@ -2150,23 +2147,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="129" t="s">
+      <c r="A1" s="130" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="131"/>
-      <c r="D1" s="131"/>
-      <c r="E1" s="131"/>
-      <c r="F1" s="131"/>
-      <c r="G1" s="131"/>
-      <c r="H1" s="131"/>
-      <c r="I1" s="131"/>
-      <c r="J1" s="131"/>
-      <c r="K1" s="131"/>
-      <c r="L1" s="131"/>
-      <c r="M1" s="131"/>
-      <c r="N1" s="131"/>
-      <c r="O1" s="132"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="132"/>
+      <c r="D1" s="132"/>
+      <c r="E1" s="132"/>
+      <c r="F1" s="132"/>
+      <c r="G1" s="132"/>
+      <c r="H1" s="132"/>
+      <c r="I1" s="132"/>
+      <c r="J1" s="132"/>
+      <c r="K1" s="132"/>
+      <c r="L1" s="132"/>
+      <c r="M1" s="132"/>
+      <c r="N1" s="132"/>
+      <c r="O1" s="133"/>
       <c r="P1" s="90"/>
       <c r="Q1" s="70"/>
     </row>
@@ -2175,7 +2172,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="125" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C2" s="72" t="s">
         <v>1</v>
@@ -2190,7 +2187,7 @@
         <v>4</v>
       </c>
       <c r="G2" s="72" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H2" s="72" t="s">
         <v>15</v>
@@ -2227,29 +2224,29 @@
       <c r="A3" s="127">
         <v>1</v>
       </c>
-      <c r="B3" s="134" t="s">
-        <v>227</v>
+      <c r="B3" s="135" t="s">
+        <v>226</v>
       </c>
       <c r="C3" s="112" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F3" s="56" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H3" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J3" s="15">
         <v>2</v>
@@ -2281,27 +2278,27 @@
       <c r="A4" s="127">
         <v>2</v>
       </c>
-      <c r="B4" s="137"/>
+      <c r="B4" s="138"/>
       <c r="C4" s="113" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D4" s="50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E4" s="50" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G4" s="50" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I4" s="50" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J4" s="38">
         <v>6</v>
@@ -2333,27 +2330,27 @@
       <c r="A5" s="11">
         <v>3</v>
       </c>
-      <c r="B5" s="137"/>
+      <c r="B5" s="138"/>
       <c r="C5" s="114" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F5" s="57" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J5" s="21">
         <v>2</v>
@@ -2385,27 +2382,27 @@
       <c r="A6" s="127">
         <v>4</v>
       </c>
-      <c r="B6" s="137"/>
+      <c r="B6" s="138"/>
       <c r="C6" s="114" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F6" s="57" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I6" s="19" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J6" s="21">
         <v>11</v>
@@ -2437,27 +2434,27 @@
       <c r="A7" s="127">
         <v>5</v>
       </c>
-      <c r="B7" s="137"/>
+      <c r="B7" s="138"/>
       <c r="C7" s="114" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F7" s="57" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="J7" s="21">
         <v>10</v>
@@ -2489,27 +2486,27 @@
       <c r="A8" s="127">
         <v>6</v>
       </c>
-      <c r="B8" s="137"/>
+      <c r="B8" s="138"/>
       <c r="C8" s="114" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F8" s="57" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I8" s="19" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J8" s="21">
         <v>1</v>
@@ -2541,27 +2538,27 @@
       <c r="A9" s="127">
         <v>7</v>
       </c>
-      <c r="B9" s="137"/>
+      <c r="B9" s="138"/>
       <c r="C9" s="114" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F9" s="57" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I9" s="19" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J9" s="21">
         <v>1</v>
@@ -2593,27 +2590,27 @@
       <c r="A10" s="127">
         <v>8</v>
       </c>
-      <c r="B10" s="137"/>
+      <c r="B10" s="138"/>
       <c r="C10" s="114" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F10" s="57" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I10" s="19" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J10" s="21">
         <v>1</v>
@@ -2645,27 +2642,27 @@
       <c r="A11" s="127">
         <v>9</v>
       </c>
-      <c r="B11" s="137"/>
+      <c r="B11" s="138"/>
       <c r="C11" s="114" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F11" s="57" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H11" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I11" s="19" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="J11" s="21">
         <v>1</v>
@@ -2697,27 +2694,27 @@
       <c r="A12" s="127">
         <v>10</v>
       </c>
-      <c r="B12" s="137"/>
+      <c r="B12" s="138"/>
       <c r="C12" s="114" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F12" s="57" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H12" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I12" s="19" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J12" s="21">
         <v>2</v>
@@ -2749,27 +2746,27 @@
       <c r="A13" s="127">
         <v>11</v>
       </c>
-      <c r="B13" s="137"/>
+      <c r="B13" s="138"/>
       <c r="C13" s="115" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D13" s="43" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E13" s="43" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F13" s="74" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G13" s="43" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H13" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I13" s="43" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J13" s="44">
         <v>1</v>
@@ -2802,28 +2799,28 @@
         <v>12</v>
       </c>
       <c r="B14" s="64" t="s">
+        <v>234</v>
+      </c>
+      <c r="C14" s="116" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="E14" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" s="59" t="s">
         <v>235</v>
       </c>
-      <c r="C14" s="116" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="32" t="s">
-        <v>83</v>
-      </c>
-      <c r="E14" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="F14" s="59" t="s">
-        <v>236</v>
-      </c>
       <c r="G14" s="32" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H14" s="76" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I14" s="32" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="J14" s="33">
         <v>2</v>
@@ -2855,29 +2852,29 @@
       <c r="A15" s="127">
         <v>13</v>
       </c>
-      <c r="B15" s="134" t="s">
-        <v>229</v>
+      <c r="B15" s="135" t="s">
+        <v>228</v>
       </c>
       <c r="C15" s="123" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D15" s="55" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E15" s="55" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F15" s="124" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G15" s="55" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H15" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I15" s="55" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J15" s="36">
         <v>1</v>
@@ -2909,27 +2906,27 @@
       <c r="A16" s="127">
         <v>14</v>
       </c>
-      <c r="B16" s="135"/>
+      <c r="B16" s="136"/>
       <c r="C16" s="114" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F16" s="57" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G16" s="19" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H16" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I16" s="19" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="J16" s="21">
         <v>1</v>
@@ -2961,27 +2958,27 @@
       <c r="A17" s="127">
         <v>5</v>
       </c>
-      <c r="B17" s="136"/>
+      <c r="B17" s="137"/>
       <c r="C17" s="117" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E17" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F17" s="58" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G17" s="28" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H17" s="53" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I17" s="28" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J17" s="29">
         <v>1</v>
@@ -3017,25 +3014,25 @@
         <v>20</v>
       </c>
       <c r="C18" s="116" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F18" s="59" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G18" s="32" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H18" s="54" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I18" s="32" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J18" s="33">
         <v>1</v>
@@ -3068,28 +3065,28 @@
         <v>17</v>
       </c>
       <c r="B19" s="64" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C19" s="116" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F19" s="59" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G19" s="32" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H19" s="54" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I19" s="32" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J19" s="33">
         <v>1</v>
@@ -3121,29 +3118,29 @@
       <c r="A20" s="127">
         <v>18</v>
       </c>
-      <c r="B20" s="134" t="s">
-        <v>231</v>
+      <c r="B20" s="135" t="s">
+        <v>230</v>
       </c>
       <c r="C20" s="112" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F20" s="56" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H20" s="55" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="J20" s="15">
         <v>2</v>
@@ -3175,27 +3172,27 @@
       <c r="A21" s="127">
         <v>19</v>
       </c>
-      <c r="B21" s="137"/>
+      <c r="B21" s="138"/>
       <c r="C21" s="114" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F21" s="57" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H21" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I21" s="19" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="J21" s="21">
         <v>1</v>
@@ -3227,27 +3224,27 @@
       <c r="A22" s="127">
         <v>20</v>
       </c>
-      <c r="B22" s="137"/>
+      <c r="B22" s="138"/>
       <c r="C22" s="114" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D22" s="19" t="s">
         <v>21</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F22" s="57" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H22" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I22" s="19" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J22" s="21">
         <v>1</v>
@@ -3279,27 +3276,27 @@
       <c r="A23" s="127">
         <v>21</v>
       </c>
-      <c r="B23" s="137"/>
+      <c r="B23" s="138"/>
       <c r="C23" s="114" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F23" s="57" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H23" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I23" s="19" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J23" s="21">
         <v>1</v>
@@ -3331,27 +3328,27 @@
       <c r="A24" s="127">
         <v>22</v>
       </c>
-      <c r="B24" s="137"/>
+      <c r="B24" s="138"/>
       <c r="C24" s="114" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D24" s="19" t="s">
         <v>22</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F24" s="57" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H24" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I24" s="19" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J24" s="21">
         <v>1</v>
@@ -3383,27 +3380,27 @@
       <c r="A25" s="127">
         <v>23</v>
       </c>
-      <c r="B25" s="137"/>
+      <c r="B25" s="138"/>
       <c r="C25" s="114" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F25" s="57" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H25" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I25" s="19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J25" s="21">
         <v>2</v>
@@ -3435,27 +3432,27 @@
       <c r="A26" s="127">
         <v>24</v>
       </c>
-      <c r="B26" s="137"/>
+      <c r="B26" s="138"/>
       <c r="C26" s="114" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F26" s="57" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H26" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I26" s="19" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J26" s="21">
         <v>2</v>
@@ -3487,27 +3484,27 @@
       <c r="A27" s="127">
         <v>25</v>
       </c>
-      <c r="B27" s="137"/>
+      <c r="B27" s="138"/>
       <c r="C27" s="114" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F27" s="57" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H27" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I27" s="19" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="J27" s="21">
         <v>1</v>
@@ -3539,27 +3536,27 @@
       <c r="A28" s="127">
         <v>26</v>
       </c>
-      <c r="B28" s="137"/>
+      <c r="B28" s="138"/>
       <c r="C28" s="114" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F28" s="57" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H28" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I28" s="19" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="J28" s="21">
         <v>3</v>
@@ -3591,27 +3588,27 @@
       <c r="A29" s="127">
         <v>27</v>
       </c>
-      <c r="B29" s="137"/>
+      <c r="B29" s="138"/>
       <c r="C29" s="114" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F29" s="60" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G29" s="60" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H29" s="60" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I29" s="60" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J29" s="61">
         <v>1</v>
@@ -3621,7 +3618,7 @@
         <v>5</v>
       </c>
       <c r="L29" s="12" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="M29" s="23">
         <v>0.1</v>
@@ -3638,34 +3635,34 @@
         <v>0.5</v>
       </c>
       <c r="Q29" s="107" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="127">
         <v>28</v>
       </c>
-      <c r="B30" s="137"/>
+      <c r="B30" s="138"/>
       <c r="C30" s="114" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I30" s="19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J30" s="21">
         <v>5</v>
@@ -3697,27 +3694,27 @@
       <c r="A31" s="127">
         <v>29</v>
       </c>
-      <c r="B31" s="137"/>
+      <c r="B31" s="138"/>
       <c r="C31" s="114" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F31" s="57" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H31" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I31" s="19" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J31" s="21">
         <v>1</v>
@@ -3749,27 +3746,27 @@
       <c r="A32" s="127">
         <v>30</v>
       </c>
-      <c r="B32" s="137"/>
+      <c r="B32" s="138"/>
       <c r="C32" s="114" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F32" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H32" s="38" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I32" s="19" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="J32" s="21">
         <v>1</v>
@@ -3801,27 +3798,27 @@
       <c r="A33" s="127">
         <v>31</v>
       </c>
-      <c r="B33" s="137"/>
+      <c r="B33" s="138"/>
       <c r="C33" s="114" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E33" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F33" s="57" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G33" s="19" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H33" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I33" s="19" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J33" s="21">
         <v>1</v>
@@ -3853,27 +3850,27 @@
       <c r="A34" s="127">
         <v>32</v>
       </c>
-      <c r="B34" s="138"/>
+      <c r="B34" s="139"/>
       <c r="C34" s="117" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D34" s="28" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E34" s="28" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F34" s="58" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G34" s="28" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H34" s="53" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I34" s="28" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="J34" s="29">
         <v>1</v>
@@ -3906,28 +3903,28 @@
         <v>33</v>
       </c>
       <c r="B35" s="77" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C35" s="118" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D35" s="78" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E35" s="78" t="s">
+        <v>243</v>
+      </c>
+      <c r="F35" s="79" t="s">
+        <v>133</v>
+      </c>
+      <c r="G35" s="78" t="s">
+        <v>207</v>
+      </c>
+      <c r="H35" s="80" t="s">
+        <v>249</v>
+      </c>
+      <c r="I35" s="78" t="s">
         <v>244</v>
-      </c>
-      <c r="F35" s="79" t="s">
-        <v>134</v>
-      </c>
-      <c r="G35" s="78" t="s">
-        <v>208</v>
-      </c>
-      <c r="H35" s="80" t="s">
-        <v>250</v>
-      </c>
-      <c r="I35" s="78" t="s">
-        <v>245</v>
       </c>
       <c r="J35" s="81">
         <v>1</v>
@@ -3959,29 +3956,29 @@
       <c r="A36" s="127">
         <v>34</v>
       </c>
-      <c r="B36" s="134" t="s">
-        <v>233</v>
+      <c r="B36" s="135" t="s">
+        <v>232</v>
       </c>
       <c r="C36" s="112" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D36" s="13" t="s">
         <v>6</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F36" s="56" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H36" s="55" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I36" s="13" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J36" s="15">
         <v>1</v>
@@ -4013,27 +4010,27 @@
       <c r="A37" s="127">
         <v>35</v>
       </c>
-      <c r="B37" s="137"/>
+      <c r="B37" s="138"/>
       <c r="C37" s="114" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E37" s="19" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F37" s="57" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H37" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I37" s="19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J37" s="21">
         <v>1</v>
@@ -4065,27 +4062,27 @@
       <c r="A38" s="127">
         <v>36</v>
       </c>
-      <c r="B38" s="137"/>
+      <c r="B38" s="138"/>
       <c r="C38" s="113" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D38" s="50" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E38" s="50" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F38" s="24" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G38" s="50" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H38" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I38" s="50" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J38" s="38">
         <v>1</v>
@@ -4117,27 +4114,27 @@
       <c r="A39" s="127">
         <v>37</v>
       </c>
-      <c r="B39" s="137"/>
+      <c r="B39" s="138"/>
       <c r="C39" s="114" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E39" s="19" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F39" s="57" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G39" s="19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H39" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I39" s="19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J39" s="21">
         <v>1</v>
@@ -4169,27 +4166,27 @@
       <c r="A40" s="127">
         <v>38</v>
       </c>
-      <c r="B40" s="137"/>
+      <c r="B40" s="138"/>
       <c r="C40" s="114" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F40" s="57" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H40" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I40" s="19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J40" s="21">
         <v>1</v>
@@ -4221,27 +4218,27 @@
       <c r="A41" s="127">
         <v>39</v>
       </c>
-      <c r="B41" s="137"/>
+      <c r="B41" s="138"/>
       <c r="C41" s="114" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D41" s="19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E41" s="19" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F41" s="57" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G41" s="21" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H41" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I41" s="19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J41" s="21">
         <v>1</v>
@@ -4251,50 +4248,50 @@
         <v>5</v>
       </c>
       <c r="L41" s="40" t="s">
-        <v>239</v>
-      </c>
-      <c r="M41" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="N41" s="62" t="e">
+        <v>238</v>
+      </c>
+      <c r="M41" s="23">
+        <v>0.36699999999999999</v>
+      </c>
+      <c r="N41" s="62">
         <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O41" s="98" t="s">
-        <v>24</v>
+        <v>0.36699999999999999</v>
+      </c>
+      <c r="O41" s="98">
+        <v>0.36699999999999999</v>
       </c>
       <c r="P41" s="92">
         <v>7.34</v>
       </c>
       <c r="Q41" s="107" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="42" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="127">
         <v>40</v>
       </c>
-      <c r="B42" s="138"/>
+      <c r="B42" s="139"/>
       <c r="C42" s="117" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D42" s="28" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E42" s="28" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F42" s="58" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G42" s="28" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H42" s="53" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I42" s="28" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J42" s="29">
         <v>1</v>
@@ -4304,7 +4301,7 @@
         <v>5</v>
       </c>
       <c r="L42" s="41" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="M42" s="31">
         <v>0.71</v>
@@ -4327,28 +4324,28 @@
         <v>41</v>
       </c>
       <c r="B43" s="77" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C43" s="118" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D43" s="78" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E43" s="78" t="s">
+        <v>243</v>
+      </c>
+      <c r="F43" s="79" t="s">
+        <v>140</v>
+      </c>
+      <c r="G43" s="78" t="s">
+        <v>222</v>
+      </c>
+      <c r="H43" s="80" t="s">
+        <v>249</v>
+      </c>
+      <c r="I43" s="78" t="s">
         <v>244</v>
-      </c>
-      <c r="F43" s="79" t="s">
-        <v>141</v>
-      </c>
-      <c r="G43" s="78" t="s">
-        <v>223</v>
-      </c>
-      <c r="H43" s="80" t="s">
-        <v>250</v>
-      </c>
-      <c r="I43" s="78" t="s">
-        <v>245</v>
       </c>
       <c r="J43" s="81">
         <v>1</v>
@@ -4380,29 +4377,29 @@
       <c r="A44" s="127">
         <v>42</v>
       </c>
-      <c r="B44" s="139" t="s">
-        <v>228</v>
+      <c r="B44" s="140" t="s">
+        <v>227</v>
       </c>
       <c r="C44" s="112" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E44" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="F44" s="56" t="s">
+        <v>119</v>
+      </c>
+      <c r="G44" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="H44" s="55" t="s">
+        <v>249</v>
+      </c>
+      <c r="I44" s="13" t="s">
         <v>244</v>
-      </c>
-      <c r="F44" s="56" t="s">
-        <v>120</v>
-      </c>
-      <c r="G44" s="13" t="s">
-        <v>210</v>
-      </c>
-      <c r="H44" s="55" t="s">
-        <v>250</v>
-      </c>
-      <c r="I44" s="13" t="s">
-        <v>245</v>
       </c>
       <c r="J44" s="15">
         <v>1</v>
@@ -4434,27 +4431,27 @@
       <c r="A45" s="127">
         <v>43</v>
       </c>
-      <c r="B45" s="140"/>
+      <c r="B45" s="141"/>
       <c r="C45" s="114" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D45" s="19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E45" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="F45" s="57" t="s">
+        <v>122</v>
+      </c>
+      <c r="G45" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="H45" s="50" t="s">
+        <v>249</v>
+      </c>
+      <c r="I45" s="19" t="s">
         <v>244</v>
-      </c>
-      <c r="F45" s="57" t="s">
-        <v>123</v>
-      </c>
-      <c r="G45" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="H45" s="50" t="s">
-        <v>250</v>
-      </c>
-      <c r="I45" s="19" t="s">
-        <v>245</v>
       </c>
       <c r="J45" s="21">
         <v>1</v>
@@ -4486,27 +4483,27 @@
       <c r="A46" s="127">
         <v>44</v>
       </c>
-      <c r="B46" s="140"/>
+      <c r="B46" s="141"/>
       <c r="C46" s="114" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D46" s="19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E46" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="F46" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="G46" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="H46" s="50" t="s">
+        <v>249</v>
+      </c>
+      <c r="I46" s="19" t="s">
         <v>244</v>
-      </c>
-      <c r="F46" s="19" t="s">
-        <v>124</v>
-      </c>
-      <c r="G46" s="19" t="s">
-        <v>212</v>
-      </c>
-      <c r="H46" s="50" t="s">
-        <v>250</v>
-      </c>
-      <c r="I46" s="19" t="s">
-        <v>245</v>
       </c>
       <c r="J46" s="21">
         <v>1</v>
@@ -4533,34 +4530,34 @@
         <v>5.9499999999999993</v>
       </c>
       <c r="Q46" s="108" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="47" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="127">
         <v>45</v>
       </c>
-      <c r="B47" s="140"/>
+      <c r="B47" s="141"/>
       <c r="C47" s="119" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D47" s="66" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E47" s="66" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F47" s="66" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G47" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H47" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I47" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="J47" s="67">
         <v>2</v>
@@ -4570,49 +4567,49 @@
         <v>10</v>
       </c>
       <c r="L47" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="M47" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="N47" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="O47" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="P47" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="Q47" s="109" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="48" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="127">
         <v>46</v>
       </c>
-      <c r="B48" s="140"/>
+      <c r="B48" s="141"/>
       <c r="C48" s="65" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D48" s="66" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E48" s="66" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F48" s="66" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G48" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H48" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I48" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="J48" s="67">
         <v>1</v>
@@ -4622,49 +4619,49 @@
         <v>5</v>
       </c>
       <c r="L48" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="M48" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="N48" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="O48" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="P48" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="Q48" s="109" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="49" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="127">
         <v>47</v>
       </c>
-      <c r="B49" s="141"/>
+      <c r="B49" s="142"/>
       <c r="C49" s="120" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D49" s="86" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E49" s="86" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F49" s="86" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G49" s="86" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H49" s="87" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I49" s="86" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="J49" s="88">
         <v>1</v>
@@ -4674,22 +4671,22 @@
         <v>5</v>
       </c>
       <c r="L49" s="86" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="M49" s="86" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="N49" s="86" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="O49" s="86" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="P49" s="86" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="Q49" s="110" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="50" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -4702,17 +4699,17 @@
       <c r="G50" s="5"/>
       <c r="H50" s="5"/>
       <c r="I50"/>
-      <c r="J50" s="133" t="s">
+      <c r="J50" s="134" t="s">
         <v>7</v>
       </c>
-      <c r="K50" s="133"/>
-      <c r="L50" s="133"/>
-      <c r="M50" s="133"/>
+      <c r="K50" s="134"/>
+      <c r="L50" s="134"/>
+      <c r="M50" s="134"/>
       <c r="N50" s="2"/>
       <c r="O50" s="5"/>
       <c r="P50" s="3">
-        <f>SUM(P3:P16)</f>
-        <v>35.359000000000002</v>
+        <f>SUM(P3:P49)</f>
+        <v>139.57899999999998</v>
       </c>
       <c r="Q50" s="5"/>
     </row>
@@ -4726,20 +4723,20 @@
       <c r="G51" s="5"/>
       <c r="H51" s="5"/>
       <c r="I51"/>
-      <c r="J51" s="128" t="s">
+      <c r="J51" s="129" t="s">
         <v>11</v>
       </c>
-      <c r="K51" s="128"/>
-      <c r="L51" s="128"/>
-      <c r="M51" s="128"/>
+      <c r="K51" s="129"/>
+      <c r="L51" s="129"/>
+      <c r="M51" s="129"/>
       <c r="N51" s="4">
-        <f>SUM(N3:N16)</f>
-        <v>9.4210000000000012</v>
+        <f>SUM(N3:N49)</f>
+        <v>29.879000000000001</v>
       </c>
       <c r="O51" s="5"/>
-      <c r="P51" s="142">
+      <c r="P51" s="128">
         <f>P50/5</f>
-        <v>7.0718000000000005</v>
+        <v>27.915799999999997</v>
       </c>
       <c r="Q51" s="5"/>
     </row>

</xml_diff>